<commit_message>
update delivery example options
</commit_message>
<xml_diff>
--- a/static/excel/pool-importvorlage-komplett.xlsx
+++ b/static/excel/pool-importvorlage-komplett.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alpinpool.sharepoint.com/sites/dm/Freigegebene Dokumente/30-39 Tools Intern/32 Applications/32.01 Retype/pool-docu/datamgmt_docs/static/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alpinpool.sharepoint.com/sites/dm/Freigegebene Dokumente/30-39 Tools Intern/32 Applications/32.01 Retype/edi-docs/static/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{E62174D8-0D03-0C4E-AC03-7E0C00DB33D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA19EA30-108F-7649-87A7-E86701F3FFC6}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E62174D8-0D03-0C4E-AC03-7E0C00DB33D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{946C66F8-581B-904B-A7B1-E8549C8197D9}"/>
   <bookViews>
     <workbookView xWindow="54160" yWindow="620" windowWidth="34140" windowHeight="19440" xr2:uid="{D7DA82DE-661B-4434-8FCB-AD97B6E46B4F}"/>
   </bookViews>
@@ -239,9 +239,6 @@
     <t>Alternative →</t>
   </si>
   <si>
-    <t>available,not_available,on_request,tracked</t>
-  </si>
-  <si>
     <t>wenn 'tracked' zb 5</t>
   </si>
   <si>
@@ -288,6 +285,9 @@
   </si>
   <si>
     <t>Material=Stahl|Länge=10mm</t>
+  </si>
+  <si>
+    <t>available,not_available,on_request,tracked,available_no_delivery_date</t>
   </si>
 </sst>
 </file>
@@ -344,7 +344,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -360,9 +360,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -400,7 +400,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -506,7 +506,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -673,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -712,7 +712,7 @@
         <v>12</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>13</v>
@@ -757,7 +757,7 @@
         <v>26</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AE1" s="1" t="s">
         <v>27</v>
@@ -817,13 +817,13 @@
         <v>45</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AY1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="BA1" s="1" t="s">
         <v>46</v>
@@ -840,10 +840,10 @@
         <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>50</v>
@@ -915,7 +915,7 @@
         <v>58</v>
       </c>
       <c r="AD2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AE2" t="s">
         <v>59</v>
@@ -945,31 +945,31 @@
         <v>66</v>
       </c>
       <c r="AR2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AT2" t="s">
         <v>83</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>67</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AV2" t="s">
         <v>68</v>
       </c>
-      <c r="AV2" t="s">
-        <v>69</v>
-      </c>
       <c r="AW2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AX2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AY2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AZ2" t="s">
         <v>77</v>
       </c>
-      <c r="AZ2" t="s">
-        <v>78</v>
-      </c>
       <c r="BA2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="BB2" s="3">
         <v>45170</v>
@@ -985,17 +985,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA0AE64D09535C45B43E32951E7FE192" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e92b413ad24d189239e7f487050cfd98">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="972a4302-61b6-4e60-8451-b9c9ef50fbef" xmlns:ns3="c9de2a3f-a2ad-4682-ba79-07e79da285ff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e98146d495d482b07aa7e65b34436cf8" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA0AE64D09535C45B43E32951E7FE192" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="489853e32009d160672205dd7ef2dc70">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="972a4302-61b6-4e60-8451-b9c9ef50fbef" xmlns:ns3="c9de2a3f-a2ad-4682-ba79-07e79da285ff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a85cd6d35e0f0f99e00eb81bbf9e5a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="972a4302-61b6-4e60-8451-b9c9ef50fbef"/>
     <xsd:import namespace="c9de2a3f-a2ad-4682-ba79-07e79da285ff"/>
     <xsd:element name="properties">
@@ -1236,7 +1227,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c9de2a3f-a2ad-4682-ba79-07e79da285ff" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="972a4302-61b6-4e60-8451-b9c9ef50fbef">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notiz xmlns="972a4302-61b6-4e60-8451-b9c9ef50fbef" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A336D5E-FFEC-450C-B51E-00B0CBD27DF7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEF06674-B273-439D-B6E9-31FC69439600}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1244,21 +1260,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01557CEC-DCF7-4A3B-8D41-7BEE3FF06D01}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="972a4302-61b6-4e60-8451-b9c9ef50fbef"/>
-    <ds:schemaRef ds:uri="c9de2a3f-a2ad-4682-ba79-07e79da285ff"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57322F88-4DA0-49B5-A109-49FFD45868CD}"/>
 </file>
</xml_diff>